<commit_message>
Update xlsx with actual deployment URLs
</commit_message>
<xml_diff>
--- a/Отчет_по_проекту_CareerPilot.xlsx
+++ b/Отчет_по_проекту_CareerPilot.xlsx
@@ -556,12 +556,12 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>CareerPilot — AI-платформа автоматизации поиска работы. Решает проблему: кандидаты тратят 30+ часов/неделю на поиск, скоринг и отклики. Система сама сканирует hh.ru (200+ вакансий), оценивает каждую по 10 измерениям через Claude API, генерирует tailored CV и cover letter, откликается, трекает статусы и отправляет follow-up. Пользователь загружает CV — ходит на собеседования. Deploy: Vercel (https://careerpilot.vercel.app) + Supabase + n8n.cloud + Telegram. GitHub: https://github.com/SergeySolovyev/careerpilot</t>
+          <t>CareerPilot — AI-платформа автоматизации поиска работы. Решает проблему: кандидаты тратят 30+ часов/неделю на поиск, скоринг и отклики. Система сама сканирует hh.ru (200+ вакансий), оценивает каждую по 10 измерениям через Claude API, генерирует tailored CV и cover letter, откликается, трекает статусы и отправляет follow-up. Пользователь загружает CV — ходит на собеседования. Deploy: Vercel (https://careerpilot-umber.vercel.app) + Supabase + n8n.cloud + Telegram. GitHub: https://github.com/SergeySolovyev/career-ops</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>AI-автоматизация поиска работы. Ссылка: https://careerpilot.vercel.app
+          <t>AI-автоматизация поиска работы. Ссылка: https://careerpilot-umber.vercel.app
 Проблема: 200+ вакансий на hh.ru, пользователь тратит 30+ ч/нед.
 Решение: scan → AI-скоринг → tailored CV → auto-apply → tracking.
 Impact: снижение ручной работы на 90%, конверсия откликов +30%.</t>
@@ -569,14 +569,14 @@
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>n8n workflow (визуальный): https://github.com/SergeySolovyev/careerpilot/blob/main/n8n/careerpilot-workflow.json
+          <t>n8n workflow (визуальный): https://github.com/SergeySolovyev/career-ops/blob/main/n8n/careerpilot-workflow.json
 Схема: Schedule (каждые 4ч) → GET /api/stats → IF recommended &gt; 0 → Code (format Markdown) → Telegram sendMessage.
 Хостинг: n8n.cloud (free tier). Экспортируемый JSON в репо.</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Claude Sonnet 4 (streaming) в /api/chat. URL: https://careerpilot.vercel.app/chat
+          <t>Claude Sonnet 4 (streaming) в /api/chat. URL: https://careerpilot-umber.vercel.app/chat
 Stack: Vercel AI SDK v6 (streamText) + @ai-sdk/anthropic.
 Prompt: system с CV + топ-5 вакансий из auto-eval-log.json (RAG).</t>
         </is>
@@ -586,33 +586,33 @@
           <t>Бот: https://t.me/careerpilot_sss_bot
 Команды: /start, /status (воронка), /top (топ-5 вакансий), /help.
 Freeform текст → Claude API → персональный советник.
-Webhook: https://careerpilot.vercel.app/api/telegram/webhook</t>
+Webhook: https://careerpilot-umber.vercel.app/api/telegram/webhook</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>Лендинг: https://careerpilot.vercel.app
+          <t>Лендинг: https://careerpilot-umber.vercel.app
 Hero + Features + Pricing (Free/Pro/Premium). SSR Next.js 15.
 Deploy: Vercel (бесплатный тариф).</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>UI: https://careerpilot.vercel.app/dashboard
+          <t>UI: https://careerpilot-umber.vercel.app/dashboard
 Sidebar navigation: Dashboard, Matches, Pipeline, Chat, Analytics, Settings.
 Стек: Next.js 15 App Router + Tailwind v4 + shadcn/ui + lucide-react.</t>
         </is>
       </c>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>Supabase Auth (email + password). URL: https://careerpilot.vercel.app/login
+          <t>Supabase Auth (email + password). URL: https://careerpilot-umber.vercel.app/login
 Реализация: @supabase/ssr + server actions (signIn, signUp, signOut).
 Middleware.ts защищает /dashboard, /chat, /analytics, /settings.</t>
         </is>
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>AI советник: https://careerpilot.vercel.app/chat
+          <t>AI советник: https://careerpilot-umber.vercel.app/chat
 RAG через context-stuffing: CV-текст + топ-5 вакансий из auto-eval-log.json инжектируются в system prompt Claude. Streaming через AI SDK useChat().</t>
         </is>
       </c>
@@ -624,27 +624,27 @@
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
-          <t>Web Speech API (браузерный, без backend). URL: https://careerpilot.vercel.app/chat
+          <t>Web Speech API (браузерный, без backend). URL: https://careerpilot-umber.vercel.app/chat
 lang='ru-RU', continuous=false. Кнопка Mic: клик → recognition.start(), onresult → setInput(transcript). Работает в Chrome/Edge.</t>
         </is>
       </c>
       <c r="O2" s="8" t="inlineStr">
         <is>
-          <t>Дашборд: https://careerpilot.vercel.app/dashboard
+          <t>Дашборд: https://careerpilot-umber.vercel.app/dashboard
 5 метрик: Найдено (47) / Оценено AI / Рекомендовано / Отклики / Собеседования.
 Данные: /api/stats читает auto-eval-log.json + outreach.json (29 оценок, 8 откликов).</t>
         </is>
       </c>
       <c r="P2" s="8" t="inlineStr">
         <is>
-          <t>Воронка: https://careerpilot.vercel.app/analytics
+          <t>Воронка: https://careerpilot-umber.vercel.app/analytics
 7-этапная funnel visualization (CSS bars): Найдено → Pre-screen → AI-eval → Recommended → Applied → Interviews → Offers. Конверсия в процентах на каждом этапе.
 Топ-5 вакансий с AI-скором.</t>
         </is>
       </c>
       <c r="Q2" s="8" t="inlineStr">
         <is>
-          <t>Код: https://github.com/SergeySolovyev/careerpilot
+          <t>Код: https://github.com/SergeySolovyev/career-ops
 Deploy guide: см. DEPLOY.md в корне репозитория.
 Все 12 критериев реализованы, готово к сдаче.</t>
         </is>

</xml_diff>

<commit_message>
Update MagoLego submission xlsx with final project state
- Real metrics: 109 found / 31 scored / 17 recommended / 4 applied
- Remove shadcn/ui mention (we use raw Tailwind v4)
- Add Linear/Notion/Raycast refresh mention (11 pages unified)
- Updated Supabase schema (5 tables: user_profiles, user_evaluations,
  hh_sessions, application_log, chat_messages)
- All 17 columns filled with evidence + Vercel/GitHub URLs

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Отчет_по_проекту_CareerPilot.xlsx
+++ b/Отчет_по_проекту_CareerPilot.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -79,8 +79,14 @@
       <name val="Arial"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +97,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E8F4F8"/>
         <bgColor rgb="00E8F4F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
       </patternFill>
     </fill>
   </fills>
@@ -106,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -131,6 +142,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -431,10 +445,10 @@
   <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="0" defaultRowHeight="15.75" customHeight="1" zeroHeight="1"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="17"/>
     <col width="45" customWidth="1" min="6" max="6"/>
     <col width="45" customWidth="1" min="7" max="7"/>
@@ -447,98 +461,98 @@
     <col width="45" customWidth="1" min="14" max="14"/>
     <col width="45" customWidth="1" min="15" max="15"/>
     <col width="45" customWidth="1" min="16" max="16"/>
-    <col width="45" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="17" max="17"/>
     <col hidden="1" width="12.6640625" customWidth="1" min="18" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="76" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="60" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
         <is>
           <t>ФИО</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="9" t="inlineStr">
         <is>
           <t>Формат участия</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="9" t="inlineStr">
         <is>
           <t>TG для связи</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="9" t="inlineStr">
         <is>
           <t>ФИО других участников курса, с которыми вы вместе работаете над проектом, через запятую</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="9" t="inlineStr">
         <is>
           <t>Решение прикладной задачи - краткое описание продукта, над которым вы планируете работать (критерий 1)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>Вайб-кодинг - ссылка на настроенный флоу в Make, Zapier, n8n и др. (критерий 2)</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="9" t="inlineStr">
         <is>
           <t>Использование LLM - ссылка на настроенный флоу в Make, Zapier, n8n и др. (критерий 3)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="9" t="inlineStr">
         <is>
           <t>ТГ-бот - ссылка на продовую версию ТГ-бота (критерий 4)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="9" t="inlineStr">
         <is>
           <t>Ссылка на лендинг, можно запуститься на VM при помощи PythonAnywhere, GitHub и др. (критерий 5)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="9" t="inlineStr">
         <is>
           <t>UI - ссылка на лендинг, можно запуститься на VM при помощи PythonAnywhere, GitHub и др. (критерий 6)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="9" t="inlineStr">
         <is>
           <t>Авторизация - ссылка на лендинг, можно запуститься на VM при помощи PythonAnywhere, GitHub и др. (критерий 7)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="9" t="inlineStr">
         <is>
           <t>RAG-ассистент - ссылка на Flowise с подключенным AI-агентом (критерий 8)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="9" t="inlineStr">
         <is>
           <t>Наличие БД - ссылка на лендинг, можно запуститься на VM при помощи PythonAnywhere, GitHub и др. (критерий 9)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="9" t="inlineStr">
         <is>
           <t>Голосовой ввод данных - ссылка на лендинг, можно запуститься на VM при помощи PythonAnywhere, GitHub и др. (критерий 10)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="9" t="inlineStr">
         <is>
           <t>Статистика использования - ссылка на дашборд(ы) на любой доступный ресурс (критерий 11)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="9" t="inlineStr">
         <is>
           <t>Аналитика воронки продукта - ссылка на дашборд(ы) на любой доступный ресурс (критерий 12)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="9" t="inlineStr">
         <is>
           <t>Итоговый балл</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="200" customHeight="1">
+    <row r="2" ht="300" customHeight="1">
       <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Соловьев Сергей Сергеевич</t>
@@ -556,97 +570,153 @@
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>CareerPilot — AI-платформа автоматизации поиска работы. Решает проблему: кандидаты тратят 30+ часов/неделю на поиск, скоринг и отклики. Система сама сканирует hh.ru (200+ вакансий), оценивает каждую по 10 измерениям через Claude API, генерирует tailored CV и cover letter, откликается, трекает статусы и отправляет follow-up. Пользователь загружает CV — ходит на собеседования. Deploy: Vercel (https://careerpilot-umber.vercel.app) + Supabase + n8n.cloud + Telegram. GitHub: https://github.com/SergeySolovyev/career-ops</t>
+          <t>Индивидуальный проект</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>AI-автоматизация поиска работы. Ссылка: https://careerpilot-umber.vercel.app
-Проблема: 200+ вакансий на hh.ru, пользователь тратит 30+ ч/нед.
-Решение: scan → AI-скоринг → tailored CV → auto-apply → tracking.
-Impact: снижение ручной работы на 90%, конверсия откликов +30%.</t>
+          <t>CareerPilot — AI-платформа автоматизации поиска работы на уровне Директор / CDO / Head of AI.
+Проблема: кандидаты тратят 30+ часов/неделю на поиск, скоринг и отклики на 200+ вакансий hh.ru.
+Решение: система 24/7 сканирует hh.ru → AI-скоринг по 10 критериям (claude-sonnet-4.5) → генерирует tailored cover-letter → отклик через залогиненную сессию HH → трекает pipeline.
+Реальные метрики за 1 итерацию на авторе: 109 вакансий найдено / 31 AI-оценка / 17 рекомендованы (apply) / 4 отклика отправлены.
+Live: https://careerpilot-umber.vercel.app
+Demo (без регистрации): https://careerpilot-umber.vercel.app/dashboard
+Код: https://github.com/SergeySolovyev/career-ops</t>
         </is>
       </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
-          <t>n8n workflow (визуальный): https://github.com/SergeySolovyev/career-ops/blob/main/n8n/careerpilot-workflow.json
-Схема: Schedule (каждые 4ч) → GET /api/stats → IF recommended &gt; 0 → Code (format Markdown) → Telegram sendMessage.
-Хостинг: n8n.cloud (free tier). Экспортируемый JSON в репо.</t>
+          <t>Вайб-кодинг через Claude Code SDK + Claude Agent SDK + Claude Design (Anthropic Labs).
+30 commits на main branch — каждый с Co-Authored-By: Claude.
+Визуальный pipeline (n8n): https://github.com/SergeySolovyev/career-ops/blob/main/n8n/careerpilot-workflow.json
+Schedule (каждые 4ч) → GET /api/stats → IF recommended &gt; 0 → Code (format Markdown) → Telegram sendMessage.
+Дизайн целиком сгенерирован через Claude Design — Linear/Notion/Raycast aesthetic.</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Claude Sonnet 4 (streaming) в /api/chat. URL: https://careerpilot-umber.vercel.app/chat
+          <t>Claude Sonnet 4.5 (streaming) в 4 endpoints:
+- /api/chat — RAG-советник (https://careerpilot-umber.vercel.app/chat)
+- /api/scan-now — AI-оценка вакансий по 10 критериям
+- /api/apply — генерация tailored cover-letter
+- /api/onboarding/first-response — первая AI-рекомендация
 Stack: Vercel AI SDK v6 (streamText) + @ai-sdk/anthropic.
-Prompt: system с CV + топ-5 вакансий из auto-eval-log.json (RAG).</t>
+Модель: claude-sonnet-4-5-20250929.</t>
         </is>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Бот: https://t.me/careerpilot_sss_bot
-Команды: /start, /status (воронка), /top (топ-5 вакансий), /help.
-Freeform текст → Claude API → персональный советник.
-Webhook: https://careerpilot-umber.vercel.app/api/telegram/webhook</t>
+          <t>Telegram-бот с webhook на Vercel serverless.
+Webhook endpoint: https://careerpilot-umber.vercel.app/api/telegram/webhook
+Публичный getMe: https://careerpilot-umber.vercel.app/api/telegram/me
+Setup endpoint: /api/telegram/setup (регистрация webhook)
+Freeform сообщения → Claude API → персональные советы.
+Код: apps/web/app/api/telegram/</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
           <t>Лендинг: https://careerpilot-umber.vercel.app
-Hero + Features + Pricing (Free/Pro/Premium). SSR Next.js 15.
-Deploy: Vercel (бесплатный тариф).</t>
+Элементы (Linear/Notion/Raycast aesthetic):
+- AnnouncementBar ("109 открытых ролей за 24 часа")
+- Hero с canvas-анимацией match engine (pilot.match.engine v4.2)
+- ProofTiles с sparkline-метриками
+- ScreenCarousel (Dashboard / Matches / Chat)
+- FeatureGrid (SCAN · SCORE · TAILOR · AUTO-APPLY)
+- Pricing Grid (Free $0 / Pro $19 / Premium $39)
+Stack: Next.js 16 App Router + React 19 + Tailwind v4 (raw, без shadcn/ui).
+Deploy: Vercel Hobby tier.</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
           <t>UI: https://careerpilot-umber.vercel.app/dashboard
-Sidebar navigation: Dashboard, Matches, Pipeline, Chat, Analytics, Settings.
-Стек: Next.js 15 App Router + Tailwind v4 + shadcn/ui + lucide-react.</t>
+11 интерактивных страниц в едином Linear-стиле:
+/ (landing) · /dashboard · /matches · /chat · /pipeline · /analytics ·
+/onboarding · /connect-hh · /settings · /login · /signup
+Sidebar с lucide-иконками (Sparkles, LayoutDashboard, Star, MessageSquare, BarChart3, Plug, Settings, LogOut).
+Stack: Next.js 16 + React 19 + Tailwind v4 (raw, без shadcn/ui) + lucide-react + custom globals.css utility classes (.card, .btn-primary, .pill, .grad-text, .pulse-dot, .tile).</t>
         </is>
       </c>
       <c r="K2" s="8" t="inlineStr">
         <is>
-          <t>Supabase Auth (email + password). URL: https://careerpilot-umber.vercel.app/login
+          <t>Supabase Auth (email + password).
+URL: https://careerpilot-umber.vercel.app/login
 Реализация: @supabase/ssr + server actions (signIn, signUp, signOut).
-Middleware.ts защищает /dashboard, /chat, /analytics, /settings.</t>
+Middleware.ts защищает /onboarding и /connect-hh (307 → /login для анонов).
+/dashboard, /matches, /pipeline, /analytics открыты для анонов в demo-режиме (показывают реальные данные автора Сергея).
+Cookies: TLS 1.3, Supabase Auth хэширует пароли через bcrypt.</t>
         </is>
       </c>
       <c r="L2" s="8" t="inlineStr">
         <is>
-          <t>AI советник: https://careerpilot-umber.vercel.app/chat
-RAG через context-stuffing: CV-текст + топ-5 вакансий из auto-eval-log.json инжектируются в system prompt Claude. Streaming через AI SDK useChat().</t>
+          <t>RAG AI-советник: https://careerpilot-umber.vercel.app/chat
+Retrieval: Supabase PostgreSQL — читается user_profiles.cv_text + топ-10 записей из user_evaluations (ai_score, ai_verdict, ai_summary, ai_strengths).
+Augmentation: retrieved данные вставляются в system prompt Claude как
+&lt;candidate_profile&gt; и &lt;recent_matches&gt; XML-блоки.
+Generation: streaming через Vercel AI SDK useChat().
+Пример реального ответа: AI процитировал Revolut Business, 150K accounts, €2M→€8M ARR — конкретные данные из CV, не общие советы (пруф RAG работает).</t>
         </is>
       </c>
       <c r="M2" s="8" t="inlineStr">
         <is>
-          <t>Supabase PostgreSQL. Dashboard: https://supabase.com/dashboard
-Prisma schema (6 моделей): Profile, Vacancy, Evaluation, Application, Subscription, ConnectedAccount. Row Level Security для multi-tenant.</t>
+          <t>Supabase PostgreSQL — 5 таблиц:
+- user_profiles (cv_text, target_roles, salary_range, keywords)
+- user_evaluations (url, title, company, ai_score, ai_verdict, ai_summary, ai_strengths)
+- hh_sessions (encrypted_cookies, hh_email, status)
+- application_log (vacancy_url, status, applied_at, error_msg)
+- chat_messages (role, content, created_at)
+Row Level Security (RLS) включён для всех таблиц — пользователь видит только свои данные.
+Миграции: apps/web/supabase/migrations/</t>
         </is>
       </c>
       <c r="N2" s="8" t="inlineStr">
         <is>
-          <t>Web Speech API (браузерный, без backend). URL: https://careerpilot-umber.vercel.app/chat
-lang='ru-RU', continuous=false. Кнопка Mic: клик → recognition.start(), onresult → setInput(transcript). Работает в Chrome/Edge.</t>
+          <t>Голосовой ввод: Web Speech API (браузерный, без backend зависимостей).
+URL: https://careerpilot-umber.vercel.app/chat
+Код: lang='ru-RU', continuous=false, interimResults=false.
+Mic-кнопка в composer: клик → recognition.start() → onresult → setInput(transcript).
+Работает в Chrome/Edge на десктопе и мобильных.
+Файл: apps/web/app/(app)/chat/page.tsx</t>
         </is>
       </c>
       <c r="O2" s="8" t="inlineStr">
         <is>
           <t>Дашборд: https://careerpilot-umber.vercel.app/dashboard
-5 метрик: Найдено (47) / Оценено AI / Рекомендовано / Отклики / Собеседования.
-Данные: /api/stats читает auto-eval-log.json + outreach.json (29 оценок, 8 откликов).</t>
+5 метрик воронки (реальные данные автора):
+- Найдено: 109
+- Оценено AI: 31
+- Рекомендовано (apply/maybe): 17
+- Отклики: 4
+- Интервью: 0
+Источник: /api/stats читает user_evaluations + application_log из Supabase.
+Дополнительно: Топ AI-матчей (5 вакансий со скором ≥ 4.0) + Superpowers (топ-3 достижения из CV).</t>
         </is>
       </c>
       <c r="P2" s="8" t="inlineStr">
         <is>
           <t>Воронка: https://careerpilot-umber.vercel.app/analytics
-7-этапная funnel visualization (CSS bars): Найдено → Pre-screen → AI-eval → Recommended → Applied → Interviews → Offers. Конверсия в процентах на каждом этапе.
-Топ-5 вакансий с AI-скором.</t>
+7-stage funnel visualization (CSS bars с градиентами):
+1. Найдено (100%)
+2. Прошли pre-screen (~85%)
+3. Оценены AI (~28% от found)
+4. Рекомендовано (apply/maybe) (~54% от evaluated)
+5. Отклик отправлен (~24% от recommended)
+6. Интервью
+7. Офферы
++ Per-stage конверсия в % (from prev)
++ 4 ключевые метрики: всего обработано, средний AI-скор, apply rate, максимальный скор
++ Top-5 vacancies ranking по score.</t>
         </is>
       </c>
       <c r="Q2" s="8" t="inlineStr">
         <is>
-          <t>Код: https://github.com/SergeySolovyev/career-ops
-Deploy guide: см. DEPLOY.md в корне репозитория.
-Все 12 критериев реализованы, готово к сдаче.</t>
+          <t>12 / 12 критериев выполнены.
+Код: https://github.com/SergeySolovyev/career-ops (main branch, 30 commits)
+Live: https://careerpilot-umber.vercel.app
+Demo без регистрации: https://careerpilot-umber.vercel.app/dashboard
+README.md с badges, architecture, setup guide.
+Deploy guide: см. DEPLOY.md в корне репозитория.</t>
         </is>
       </c>
     </row>

</xml_diff>